<commit_message>
Close nursery specification and template alignment gaps
</commit_message>
<xml_diff>
--- a/docs/templates/nursery-automation/equipment-data-template.xlsx
+++ b/docs/templates/nursery-automation/equipment-data-template.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" r:id="Raa9d170827b24df4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="Rbb78017c442746fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="3" r:id="Rb42554f028c64a86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="4" r:id="R247b866e8dd14d30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery profiles" sheetId="5" r:id="Rffa610388d8348f6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity standards" sheetId="6" r:id="Raf70099254fd41c9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery scope" sheetId="7" r:id="Rb4d8af0594c94881"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content links" sheetId="8" r:id="Rf4d9cbcee3df4836"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="9" r:id="Rc302e31b7e864ced"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start here" sheetId="1" r:id="R0cf5f56b649942d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Equipment" sheetId="2" r:id="R09d3dd855ed4451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Options" sheetId="3" r:id="R6ffbc5b42ed44cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Interfaces" sheetId="4" r:id="R62556d9b3f284795"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery profiles" sheetId="5" r:id="Ra88da7d80ebc4cc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Activity standards" sheetId="6" r:id="R5892a1af885e45a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Delivery scope" sheetId="7" r:id="Rc8d9ce4e8fc74dd9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Content links" sheetId="8" r:id="R519d9ff1de2a430f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evidence" sheetId="9" r:id="R34a1682ea3384e99"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -21,13 +21,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="202" formatCode="#,##0"/>
     <x:numFmt numFmtId="203" formatCode="yyyy-mm-dd"/>
+    <x:numFmt numFmtId="204" formatCode="#,##0.000"/>
   </x:numFmts>
-  <x:fonts count="9">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -76,13 +77,45 @@
       <x:color rgb="FF4B5A50"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF26372D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="11"/>
+      <x:color rgb="FF26372D"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="gray125"/>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE6EDE7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF234D35"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF1EF"/>
+      </x:patternFill>
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
@@ -117,7 +150,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="39">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -173,6 +206,52 @@
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -405,10 +484,10 @@
       <x:c r="D3" s="1"/>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
-      <x:c r="A4" s="5" t="str">
+      <x:c r="A4" s="23" t="str">
         <x:v>Template status</x:v>
       </x:c>
-      <x:c r="B4" s="5" t="str">
+      <x:c r="B4" s="23" t="str">
         <x:v>Draft for review · 22 October 2026</x:v>
       </x:c>
       <x:c r="C4" s="1"/>
@@ -555,7 +634,7 @@
         <x:v>Field dictionary</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
-        <x:v>equipment-data-template.json holds the same 151 fields, choices, units, guidance and blank records.</x:v>
+        <x:v>equipment-data-template.json holds the same 171 fields, choices, units, guidance and blank records.</x:v>
       </x:c>
       <x:c r="C19" s="1"/>
       <x:c r="D19" s="1"/>
@@ -2210,28 +2289,28 @@
       <x:c r="H4" s="7"/>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
-      <x:c r="A5" s="13" t="str">
+      <x:c r="A5" s="28" t="str">
         <x:v>Field key</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="str">
+      <x:c r="B5" s="28" t="str">
         <x:v>Field</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="str">
+      <x:c r="C5" s="28" t="str">
         <x:v>Entry</x:v>
       </x:c>
-      <x:c r="D5" s="13" t="str">
+      <x:c r="D5" s="28" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="E5" s="13" t="str">
+      <x:c r="E5" s="28" t="str">
         <x:v>Evidence state</x:v>
       </x:c>
-      <x:c r="F5" s="13" t="str">
+      <x:c r="F5" s="28" t="str">
         <x:v>Source ref</x:v>
       </x:c>
-      <x:c r="G5" s="13" t="str">
+      <x:c r="G5" s="28" t="str">
         <x:v>Synthetic example</x:v>
       </x:c>
-      <x:c r="H5" s="13" t="str">
+      <x:c r="H5" s="28" t="str">
         <x:v>Entry guidance and required condition</x:v>
       </x:c>
     </x:row>
@@ -2242,11 +2321,11 @@
       <x:c r="B6" s="14" t="str">
         <x:v>Profile ID</x:v>
       </x:c>
-      <x:c r="C6" s="19"/>
+      <x:c r="C6" s="29"/>
       <x:c r="D6" s="14" t="str"/>
-      <x:c r="E6" s="15"/>
-      <x:c r="F6" s="15"/>
-      <x:c r="G6" s="17" t="str">
+      <x:c r="E6" s="31"/>
+      <x:c r="F6" s="31"/>
+      <x:c r="G6" s="33" t="str">
         <x:v>SYN-PROFILE-001</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
@@ -2260,11 +2339,11 @@
       <x:c r="B7" s="14" t="str">
         <x:v>Profile version</x:v>
       </x:c>
-      <x:c r="C7" s="19"/>
+      <x:c r="C7" s="29"/>
       <x:c r="D7" s="14" t="str"/>
-      <x:c r="E7" s="15"/>
-      <x:c r="F7" s="15"/>
-      <x:c r="G7" s="17" t="str">
+      <x:c r="E7" s="31"/>
+      <x:c r="F7" s="31"/>
+      <x:c r="G7" s="33" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="H7" s="18" t="str">
@@ -2278,11 +2357,11 @@
       <x:c r="B8" s="14" t="str">
         <x:v>Profile attaches to</x:v>
       </x:c>
-      <x:c r="C8" s="19"/>
+      <x:c r="C8" s="29"/>
       <x:c r="D8" s="14" t="str"/>
-      <x:c r="E8" s="15"/>
-      <x:c r="F8" s="15"/>
-      <x:c r="G8" s="17" t="str">
+      <x:c r="E8" s="31"/>
+      <x:c r="F8" s="31"/>
+      <x:c r="G8" s="33" t="str">
         <x:v>System</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
@@ -2296,11 +2375,11 @@
       <x:c r="B9" s="14" t="str">
         <x:v>Attachment identity</x:v>
       </x:c>
-      <x:c r="C9" s="19"/>
+      <x:c r="C9" s="29"/>
       <x:c r="D9" s="14" t="str"/>
-      <x:c r="E9" s="15"/>
-      <x:c r="F9" s="15"/>
-      <x:c r="G9" s="17" t="str">
+      <x:c r="E9" s="31"/>
+      <x:c r="F9" s="31"/>
+      <x:c r="G9" s="33" t="str">
         <x:v>SYN-LINE-FAMILY</x:v>
       </x:c>
       <x:c r="H9" s="18" t="str">
@@ -2314,11 +2393,11 @@
       <x:c r="B10" s="14" t="str">
         <x:v>Profile owner</x:v>
       </x:c>
-      <x:c r="C10" s="19"/>
+      <x:c r="C10" s="29"/>
       <x:c r="D10" s="14" t="str"/>
-      <x:c r="E10" s="15"/>
-      <x:c r="F10" s="15"/>
-      <x:c r="G10" s="17"/>
+      <x:c r="E10" s="31"/>
+      <x:c r="F10" s="31"/>
+      <x:c r="G10" s="33"/>
       <x:c r="H10" s="18" t="str">
         <x:v>Required. Nominated owner; no assumed approval.</x:v>
       </x:c>
@@ -2330,11 +2409,11 @@
       <x:c r="B11" s="14" t="str">
         <x:v>Applicability conditions</x:v>
       </x:c>
-      <x:c r="C11" s="19"/>
+      <x:c r="C11" s="29"/>
       <x:c r="D11" s="14" t="str"/>
-      <x:c r="E11" s="15"/>
-      <x:c r="F11" s="15"/>
-      <x:c r="G11" s="17" t="str">
+      <x:c r="E11" s="31"/>
+      <x:c r="F11" s="31"/>
+      <x:c r="G11" s="33" t="str">
         <x:v>Selected connected potting line</x:v>
       </x:c>
       <x:c r="H11" s="18" t="str">
@@ -2348,11 +2427,11 @@
       <x:c r="B12" s="14" t="str">
         <x:v>Inherited profiles</x:v>
       </x:c>
-      <x:c r="C12" s="19"/>
+      <x:c r="C12" s="29"/>
       <x:c r="D12" s="14" t="str"/>
-      <x:c r="E12" s="15"/>
-      <x:c r="F12" s="15"/>
-      <x:c r="G12" s="17"/>
+      <x:c r="E12" s="31"/>
+      <x:c r="F12" s="31"/>
+      <x:c r="G12" s="33"/>
       <x:c r="H12" s="18" t="str">
         <x:v>When applicable. Exact versions with explicit precedence.</x:v>
       </x:c>
@@ -2364,11 +2443,11 @@
       <x:c r="B13" s="14" t="str">
         <x:v>Inheritance policy</x:v>
       </x:c>
-      <x:c r="C13" s="19"/>
+      <x:c r="C13" s="29"/>
       <x:c r="D13" s="14" t="str"/>
-      <x:c r="E13" s="15"/>
-      <x:c r="F13" s="15"/>
-      <x:c r="G13" s="17" t="str">
+      <x:c r="E13" s="31"/>
+      <x:c r="F13" s="31"/>
+      <x:c r="G13" s="33" t="str">
         <x:v>NoInheritance</x:v>
       </x:c>
       <x:c r="H13" s="18" t="str">
@@ -2382,11 +2461,11 @@
       <x:c r="B14" s="14" t="str">
         <x:v>Activity standard references</x:v>
       </x:c>
-      <x:c r="C14" s="19"/>
+      <x:c r="C14" s="29"/>
       <x:c r="D14" s="14" t="str"/>
-      <x:c r="E14" s="15"/>
-      <x:c r="F14" s="15"/>
-      <x:c r="G14" s="17" t="str">
+      <x:c r="E14" s="31"/>
+      <x:c r="F14" s="31"/>
+      <x:c r="G14" s="33" t="str">
         <x:v>SYN-ACT-001@1</x:v>
       </x:c>
       <x:c r="H14" s="18" t="str">
@@ -2400,11 +2479,11 @@
       <x:c r="B15" s="14" t="str">
         <x:v>Covered equipment and work</x:v>
       </x:c>
-      <x:c r="C15" s="19"/>
+      <x:c r="C15" s="29"/>
       <x:c r="D15" s="14" t="str"/>
-      <x:c r="E15" s="15"/>
-      <x:c r="F15" s="15"/>
-      <x:c r="G15" s="17" t="str">
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="33" t="str">
         <x:v>Line setup only</x:v>
       </x:c>
       <x:c r="H15" s="18" t="str">
@@ -2418,11 +2497,11 @@
       <x:c r="B16" s="14" t="str">
         <x:v>Work not covered by profile</x:v>
       </x:c>
-      <x:c r="C16" s="19"/>
+      <x:c r="C16" s="29"/>
       <x:c r="D16" s="14" t="str"/>
-      <x:c r="E16" s="15"/>
-      <x:c r="F16" s="15"/>
-      <x:c r="G16" s="17" t="str">
+      <x:c r="E16" s="31"/>
+      <x:c r="F16" s="31"/>
+      <x:c r="G16" s="33" t="str">
         <x:v>Site enabling works</x:v>
       </x:c>
       <x:c r="H16" s="18" t="str">
@@ -2436,11 +2515,11 @@
       <x:c r="B17" s="14" t="str">
         <x:v>Approved content references</x:v>
       </x:c>
-      <x:c r="C17" s="19"/>
+      <x:c r="C17" s="29"/>
       <x:c r="D17" s="14" t="str"/>
-      <x:c r="E17" s="15"/>
-      <x:c r="F17" s="15"/>
-      <x:c r="G17" s="17" t="str">
+      <x:c r="E17" s="31"/>
+      <x:c r="F17" s="31"/>
+      <x:c r="G17" s="33" t="str">
         <x:v>SYN-CLAUSE-001@1</x:v>
       </x:c>
       <x:c r="H17" s="18" t="str">
@@ -2454,11 +2533,11 @@
       <x:c r="B18" s="14" t="str">
         <x:v>Effective from</x:v>
       </x:c>
-      <x:c r="C18" s="22"/>
+      <x:c r="C18" s="30"/>
       <x:c r="D18" s="14" t="str"/>
-      <x:c r="E18" s="15"/>
-      <x:c r="F18" s="15"/>
-      <x:c r="G18" s="17"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="33"/>
       <x:c r="H18" s="18" t="str">
         <x:v>Before publication. Real date; applicable period.</x:v>
       </x:c>
@@ -2470,11 +2549,11 @@
       <x:c r="B19" s="14" t="str">
         <x:v>Effective to</x:v>
       </x:c>
-      <x:c r="C19" s="22"/>
+      <x:c r="C19" s="30"/>
       <x:c r="D19" s="14" t="str"/>
-      <x:c r="E19" s="15"/>
-      <x:c r="F19" s="15"/>
-      <x:c r="G19" s="17"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="33"/>
       <x:c r="H19" s="18" t="str">
         <x:v>When bounded. Blank means unspecified, not automatically current forever.</x:v>
       </x:c>
@@ -2484,13 +2563,13 @@
         <x:v>review_state</x:v>
       </x:c>
       <x:c r="B20" s="14" t="str">
-        <x:v>Review/publication state</x:v>
-      </x:c>
-      <x:c r="C20" s="19"/>
+        <x:v>Profile technical review</x:v>
+      </x:c>
+      <x:c r="C20" s="29"/>
       <x:c r="D20" s="14" t="str"/>
-      <x:c r="E20" s="15"/>
-      <x:c r="F20" s="15"/>
-      <x:c r="G20" s="17" t="str">
+      <x:c r="E20" s="31"/>
+      <x:c r="F20" s="31"/>
+      <x:c r="G20" s="33" t="str">
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="H20" s="18" t="str">
@@ -2504,20 +2583,53 @@
       <x:c r="B21" s="14" t="str">
         <x:v>Reviewer</x:v>
       </x:c>
-      <x:c r="C21" s="19"/>
+      <x:c r="C21" s="29"/>
       <x:c r="D21" s="14" t="str"/>
-      <x:c r="E21" s="15"/>
-      <x:c r="F21" s="15"/>
-      <x:c r="G21" s="17"/>
+      <x:c r="E21" s="31"/>
+      <x:c r="F21" s="31"/>
+      <x:c r="G21" s="33"/>
       <x:c r="H21" s="18" t="str">
         <x:v>Before publication. Actual attribution and evidence required.</x:v>
       </x:c>
     </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>company_key</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>PPO company key</x:v>
+      </x:c>
+      <x:c r="C22" s="29"/>
+      <x:c r="D22" s="14" t="str"/>
+      <x:c r="E22" s="31"/>
+      <x:c r="F22" s="31"/>
+      <x:c r="G22" s="33" t="str">
+        <x:v>SYN-COMPANY</x:v>
+      </x:c>
+      <x:c r="H22" s="18" t="str">
+        <x:v>Required. Company-scoped registry; no cross-company lookup.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="14" t="str">
+        <x:v>publication_state</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>Publication state</x:v>
+      </x:c>
+      <x:c r="C23" s="29"/>
+      <x:c r="D23" s="14" t="str"/>
+      <x:c r="E23" s="31"/>
+      <x:c r="F23" s="31"/>
+      <x:c r="G23" s="33" t="str">
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="H23" s="18" t="str">
+        <x:v>Required. Separate from technical review; an Excel entry publishes nothing.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="E6:E21">
-      <x:formula1>"Unknown,NotApplicable,Assumed,CustomerAdvised,SupplierDocumented,TrialMeasured"</x:formula1>
-    </x:dataValidation>
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="C8">
       <x:formula1>"Product,Assembly,Service,System,Project"</x:formula1>
     </x:dataValidation>
@@ -2525,7 +2637,13 @@
       <x:formula1>"Additive,Replacement,NoInheritance"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C20">
-      <x:formula1>"Draft,Pending,Reviewed,Published,Retired"</x:formula1>
+      <x:formula1>"Draft,Pending,Reviewed,Rejected"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E6:E23">
+      <x:formula1>"Unknown,NotApplicable,Assumed,CustomerAdvised,SupplierDocumented,TrialMeasured"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C23">
+      <x:formula1>"Draft,Published,Retired"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2593,28 +2711,28 @@
       <x:c r="H4" s="7"/>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
-      <x:c r="A5" s="13" t="str">
+      <x:c r="A5" s="28" t="str">
         <x:v>Field key</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="str">
+      <x:c r="B5" s="28" t="str">
         <x:v>Field</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="str">
+      <x:c r="C5" s="28" t="str">
         <x:v>Entry</x:v>
       </x:c>
-      <x:c r="D5" s="13" t="str">
+      <x:c r="D5" s="28" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="E5" s="13" t="str">
+      <x:c r="E5" s="28" t="str">
         <x:v>Evidence state</x:v>
       </x:c>
-      <x:c r="F5" s="13" t="str">
+      <x:c r="F5" s="28" t="str">
         <x:v>Source ref</x:v>
       </x:c>
-      <x:c r="G5" s="13" t="str">
+      <x:c r="G5" s="28" t="str">
         <x:v>Synthetic example</x:v>
       </x:c>
-      <x:c r="H5" s="13" t="str">
+      <x:c r="H5" s="28" t="str">
         <x:v>Entry guidance and required condition</x:v>
       </x:c>
     </x:row>
@@ -2625,11 +2743,11 @@
       <x:c r="B6" s="14" t="str">
         <x:v>Activity ID</x:v>
       </x:c>
-      <x:c r="C6" s="19"/>
+      <x:c r="C6" s="29"/>
       <x:c r="D6" s="14" t="str"/>
-      <x:c r="E6" s="15"/>
-      <x:c r="F6" s="15"/>
-      <x:c r="G6" s="17" t="str">
+      <x:c r="E6" s="31"/>
+      <x:c r="F6" s="31"/>
+      <x:c r="G6" s="33" t="str">
         <x:v>SYN-ACT-001</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
@@ -2643,11 +2761,11 @@
       <x:c r="B7" s="14" t="str">
         <x:v>Standard version</x:v>
       </x:c>
-      <x:c r="C7" s="19"/>
+      <x:c r="C7" s="29"/>
       <x:c r="D7" s="14" t="str"/>
-      <x:c r="E7" s="15"/>
-      <x:c r="F7" s="15"/>
-      <x:c r="G7" s="17" t="str">
+      <x:c r="E7" s="31"/>
+      <x:c r="F7" s="31"/>
+      <x:c r="G7" s="33" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="H7" s="18" t="str">
@@ -2661,11 +2779,11 @@
       <x:c r="B8" s="14" t="str">
         <x:v>Activity category</x:v>
       </x:c>
-      <x:c r="C8" s="19"/>
+      <x:c r="C8" s="29"/>
       <x:c r="D8" s="14" t="str"/>
-      <x:c r="E8" s="15"/>
-      <x:c r="F8" s="15"/>
-      <x:c r="G8" s="17" t="str">
+      <x:c r="E8" s="31"/>
+      <x:c r="F8" s="31"/>
+      <x:c r="G8" s="33" t="str">
         <x:v>Installation</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
@@ -2679,11 +2797,11 @@
       <x:c r="B9" s="14" t="str">
         <x:v>Activity description</x:v>
       </x:c>
-      <x:c r="C9" s="19"/>
+      <x:c r="C9" s="29"/>
       <x:c r="D9" s="14" t="str"/>
-      <x:c r="E9" s="15"/>
-      <x:c r="F9" s="15"/>
-      <x:c r="G9" s="17" t="str">
+      <x:c r="E9" s="31"/>
+      <x:c r="F9" s="31"/>
+      <x:c r="G9" s="33" t="str">
         <x:v>Synthetic machine placement</x:v>
       </x:c>
       <x:c r="H9" s="18" t="str">
@@ -2697,11 +2815,11 @@
       <x:c r="B10" s="14" t="str">
         <x:v>Technical driver key</x:v>
       </x:c>
-      <x:c r="C10" s="19"/>
+      <x:c r="C10" s="29"/>
       <x:c r="D10" s="14" t="str"/>
-      <x:c r="E10" s="15"/>
-      <x:c r="F10" s="15"/>
-      <x:c r="G10" s="17" t="str">
+      <x:c r="E10" s="31"/>
+      <x:c r="F10" s="31"/>
+      <x:c r="G10" s="33" t="str">
         <x:v>installed_machine_count</x:v>
       </x:c>
       <x:c r="H10" s="18" t="str">
@@ -2715,11 +2833,11 @@
       <x:c r="B11" s="14" t="str">
         <x:v>Driver unit</x:v>
       </x:c>
-      <x:c r="C11" s="19"/>
+      <x:c r="C11" s="29"/>
       <x:c r="D11" s="14" t="str"/>
-      <x:c r="E11" s="15"/>
-      <x:c r="F11" s="15"/>
-      <x:c r="G11" s="17" t="str">
+      <x:c r="E11" s="31"/>
+      <x:c r="F11" s="31"/>
+      <x:c r="G11" s="33" t="str">
         <x:v>each</x:v>
       </x:c>
       <x:c r="H11" s="18" t="str">
@@ -2733,11 +2851,11 @@
       <x:c r="B12" s="14" t="str">
         <x:v>Effort basis</x:v>
       </x:c>
-      <x:c r="C12" s="19"/>
+      <x:c r="C12" s="29"/>
       <x:c r="D12" s="14" t="str"/>
-      <x:c r="E12" s="15"/>
-      <x:c r="F12" s="15"/>
-      <x:c r="G12" s="17" t="str">
+      <x:c r="E12" s="31"/>
+      <x:c r="F12" s="31"/>
+      <x:c r="G12" s="33" t="str">
         <x:v>PersonHoursPerUnit</x:v>
       </x:c>
       <x:c r="H12" s="18" t="str">
@@ -2751,13 +2869,13 @@
       <x:c r="B13" s="14" t="str">
         <x:v>Standard value</x:v>
       </x:c>
-      <x:c r="C13" s="20"/>
+      <x:c r="C13" s="35"/>
       <x:c r="D13" s="14" t="str">
         <x:v>basis above</x:v>
       </x:c>
-      <x:c r="E13" s="15"/>
-      <x:c r="F13" s="15"/>
-      <x:c r="G13" s="21" t="n">
+      <x:c r="E13" s="31"/>
+      <x:c r="F13" s="31"/>
+      <x:c r="G13" s="37" t="n">
         <x:v>3</x:v>
       </x:c>
       <x:c r="H13" s="18" t="str">
@@ -2771,13 +2889,13 @@
       <x:c r="B14" s="14" t="str">
         <x:v>Fixed setup effort</x:v>
       </x:c>
-      <x:c r="C14" s="20"/>
+      <x:c r="C14" s="35"/>
       <x:c r="D14" s="14" t="str">
         <x:v>person-hour</x:v>
       </x:c>
-      <x:c r="E14" s="15"/>
-      <x:c r="F14" s="15"/>
-      <x:c r="G14" s="21" t="n">
+      <x:c r="E14" s="31"/>
+      <x:c r="F14" s="31"/>
+      <x:c r="G14" s="37" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H14" s="18" t="str">
@@ -2791,11 +2909,11 @@
       <x:c r="B15" s="14" t="str">
         <x:v>Crew composition</x:v>
       </x:c>
-      <x:c r="C15" s="19"/>
+      <x:c r="C15" s="29"/>
       <x:c r="D15" s="14" t="str"/>
-      <x:c r="E15" s="15"/>
-      <x:c r="F15" s="15"/>
-      <x:c r="G15" s="17" t="str">
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="33" t="str">
         <x:v>2 installers</x:v>
       </x:c>
       <x:c r="H15" s="18" t="str">
@@ -2809,11 +2927,11 @@
       <x:c r="B16" s="14" t="str">
         <x:v>Required role/skill</x:v>
       </x:c>
-      <x:c r="C16" s="19"/>
+      <x:c r="C16" s="29"/>
       <x:c r="D16" s="14" t="str"/>
-      <x:c r="E16" s="15"/>
-      <x:c r="F16" s="15"/>
-      <x:c r="G16" s="17" t="str">
+      <x:c r="E16" s="31"/>
+      <x:c r="F16" s="31"/>
+      <x:c r="G16" s="33" t="str">
         <x:v>Synthetic installer</x:v>
       </x:c>
       <x:c r="H16" s="18" t="str">
@@ -2827,11 +2945,11 @@
       <x:c r="B17" s="14" t="str">
         <x:v>Conditions</x:v>
       </x:c>
-      <x:c r="C17" s="19"/>
+      <x:c r="C17" s="29"/>
       <x:c r="D17" s="14" t="str"/>
-      <x:c r="E17" s="15"/>
-      <x:c r="F17" s="15"/>
-      <x:c r="G17" s="17" t="str">
+      <x:c r="E17" s="31"/>
+      <x:c r="F17" s="31"/>
+      <x:c r="G17" s="33" t="str">
         <x:v>Synthetic level-access case</x:v>
       </x:c>
       <x:c r="H17" s="18" t="str">
@@ -2845,11 +2963,11 @@
       <x:c r="B18" s="14" t="str">
         <x:v>Factors and order reference</x:v>
       </x:c>
-      <x:c r="C18" s="19"/>
+      <x:c r="C18" s="29"/>
       <x:c r="D18" s="14" t="str"/>
-      <x:c r="E18" s="15"/>
-      <x:c r="F18" s="15"/>
-      <x:c r="G18" s="17"/>
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="33"/>
       <x:c r="H18" s="18" t="str">
         <x:v>When adjusted. Factors apply only to declared portions; no universal multiplier.</x:v>
       </x:c>
@@ -2861,11 +2979,11 @@
       <x:c r="B19" s="14" t="str">
         <x:v>Minimum effort rule</x:v>
       </x:c>
-      <x:c r="C19" s="19"/>
+      <x:c r="C19" s="29"/>
       <x:c r="D19" s="14" t="str"/>
-      <x:c r="E19" s="15"/>
-      <x:c r="F19" s="15"/>
-      <x:c r="G19" s="17"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="33"/>
       <x:c r="H19" s="18" t="str">
         <x:v>When applicable. State where the minimum applies in calculation order.</x:v>
       </x:c>
@@ -2877,11 +2995,11 @@
       <x:c r="B20" s="14" t="str">
         <x:v>Rounding rule reference</x:v>
       </x:c>
-      <x:c r="C20" s="19"/>
+      <x:c r="C20" s="29"/>
       <x:c r="D20" s="14" t="str"/>
-      <x:c r="E20" s="15"/>
-      <x:c r="F20" s="15"/>
-      <x:c r="G20" s="17"/>
+      <x:c r="E20" s="31"/>
+      <x:c r="F20" s="31"/>
+      <x:c r="G20" s="33"/>
       <x:c r="H20" s="18" t="str">
         <x:v>Before calculation. Retain unrounded detail; governed precision/order.</x:v>
       </x:c>
@@ -2893,11 +3011,11 @@
       <x:c r="B21" s="14" t="str">
         <x:v>Activity coverage key</x:v>
       </x:c>
-      <x:c r="C21" s="19"/>
+      <x:c r="C21" s="29"/>
       <x:c r="D21" s="14" t="str"/>
-      <x:c r="E21" s="15"/>
-      <x:c r="F21" s="15"/>
-      <x:c r="G21" s="17" t="str">
+      <x:c r="E21" s="31"/>
+      <x:c r="F21" s="31"/>
+      <x:c r="G21" s="33" t="str">
         <x:v>SYN-INSTALL-SETUP</x:v>
       </x:c>
       <x:c r="H21" s="18" t="str">
@@ -2911,11 +3029,11 @@
       <x:c r="B22" s="14" t="str">
         <x:v>Covered component IDs</x:v>
       </x:c>
-      <x:c r="C22" s="19"/>
+      <x:c r="C22" s="29"/>
       <x:c r="D22" s="14" t="str"/>
-      <x:c r="E22" s="15"/>
-      <x:c r="F22" s="15"/>
-      <x:c r="G22" s="17" t="str">
+      <x:c r="E22" s="31"/>
+      <x:c r="F22" s="31"/>
+      <x:c r="G22" s="33" t="str">
         <x:v>SYN-EQ-001</x:v>
       </x:c>
       <x:c r="H22" s="18" t="str">
@@ -2929,11 +3047,11 @@
       <x:c r="B23" s="14" t="str">
         <x:v>Replaced activities</x:v>
       </x:c>
-      <x:c r="C23" s="19"/>
+      <x:c r="C23" s="29"/>
       <x:c r="D23" s="14" t="str"/>
-      <x:c r="E23" s="15"/>
-      <x:c r="F23" s="15"/>
-      <x:c r="G23" s="17"/>
+      <x:c r="E23" s="31"/>
+      <x:c r="F23" s="31"/>
+      <x:c r="G23" s="33"/>
       <x:c r="H23" s="18" t="str">
         <x:v>When applicable. Explicit precedence; otherwise unresolved conflict.</x:v>
       </x:c>
@@ -2945,11 +3063,11 @@
       <x:c r="B24" s="14" t="str">
         <x:v>Standard evidence source</x:v>
       </x:c>
-      <x:c r="C24" s="19"/>
+      <x:c r="C24" s="29"/>
       <x:c r="D24" s="14" t="str"/>
-      <x:c r="E24" s="15"/>
-      <x:c r="F24" s="15"/>
-      <x:c r="G24" s="17" t="str">
+      <x:c r="E24" s="31"/>
+      <x:c r="F24" s="31"/>
+      <x:c r="G24" s="33" t="str">
         <x:v>SYN-SRC-001</x:v>
       </x:c>
       <x:c r="H24" s="18" t="str">
@@ -2963,22 +3081,107 @@
       <x:c r="B25" s="14" t="str">
         <x:v>Standard review state</x:v>
       </x:c>
-      <x:c r="C25" s="19"/>
+      <x:c r="C25" s="29"/>
       <x:c r="D25" s="14" t="str"/>
-      <x:c r="E25" s="15"/>
-      <x:c r="F25" s="15"/>
-      <x:c r="G25" s="17" t="str">
+      <x:c r="E25" s="31"/>
+      <x:c r="F25" s="31"/>
+      <x:c r="G25" s="33" t="str">
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="H25" s="18" t="str">
         <x:v>Required. Excel value does not authorise publication.</x:v>
       </x:c>
     </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>company_key</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>PPO company key</x:v>
+      </x:c>
+      <x:c r="C26" s="29"/>
+      <x:c r="D26" s="14" t="str"/>
+      <x:c r="E26" s="31"/>
+      <x:c r="F26" s="31"/>
+      <x:c r="G26" s="33" t="str">
+        <x:v>SYN-COMPANY</x:v>
+      </x:c>
+      <x:c r="H26" s="18" t="str">
+        <x:v>Required. Company-scoped registry; no cross-company lookup.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="14" t="str">
+        <x:v>publication_state</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>Publication state</x:v>
+      </x:c>
+      <x:c r="C27" s="29"/>
+      <x:c r="D27" s="14" t="str"/>
+      <x:c r="E27" s="31"/>
+      <x:c r="F27" s="31"/>
+      <x:c r="G27" s="33" t="str">
+        <x:v>Draft</x:v>
+      </x:c>
+      <x:c r="H27" s="18" t="str">
+        <x:v>Required. Separate from technical review; an Excel entry publishes nothing.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>owner</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>Standards owner</x:v>
+      </x:c>
+      <x:c r="C28" s="29"/>
+      <x:c r="D28" s="14" t="str"/>
+      <x:c r="E28" s="31"/>
+      <x:c r="F28" s="31"/>
+      <x:c r="G28" s="33"/>
+      <x:c r="H28" s="18" t="str">
+        <x:v>Required. Nominated accountable owner; not inferred from workbook editor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="14" t="str">
+        <x:v>included_subactivities</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>Included subactivities</x:v>
+      </x:c>
+      <x:c r="C29" s="29"/>
+      <x:c r="D29" s="14" t="str"/>
+      <x:c r="E29" s="31"/>
+      <x:c r="F29" s="31"/>
+      <x:c r="G29" s="33" t="str">
+        <x:v>Placement and levelling</x:v>
+      </x:c>
+      <x:c r="H29" s="18" t="str">
+        <x:v>Before review. Identify exactly which work the standard covers.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="42" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>excluded_scope</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>Standard exclusions</x:v>
+      </x:c>
+      <x:c r="C30" s="29"/>
+      <x:c r="D30" s="14" t="str"/>
+      <x:c r="E30" s="31"/>
+      <x:c r="F30" s="31"/>
+      <x:c r="G30" s="33" t="str">
+        <x:v>Electrical integration excluded</x:v>
+      </x:c>
+      <x:c r="H30" s="18" t="str">
+        <x:v>Before review. Identify omitted work; blank does not confirm no exclusions.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="E6:E25">
-      <x:formula1>"Unknown,NotApplicable,Assumed,CustomerAdvised,SupplierDocumented,TrialMeasured"</x:formula1>
-    </x:dataValidation>
+  <x:dataValidations count="5">
     <x:dataValidation type="list" sqref="C8">
       <x:formula1>"Installation,Commissioning,Training,Integration,Setup,Handover,Other"</x:formula1>
     </x:dataValidation>
@@ -2986,7 +3189,13 @@
       <x:formula1>"PersonHoursPerUnit,UnitsPerPersonHour,CrewHoursPerUnit,FixedPersonHours,Manual"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C25">
-      <x:formula1>"Draft,Pending,Reviewed,Published,Retired"</x:formula1>
+      <x:formula1>"Draft,Pending,Reviewed,Rejected"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E6:E30">
+      <x:formula1>"Unknown,NotApplicable,Assumed,CustomerAdvised,SupplierDocumented,TrialMeasured"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C27">
+      <x:formula1>"Draft,Published,Retired"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3054,28 +3263,28 @@
       <x:c r="H4" s="7"/>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
-      <x:c r="A5" s="13" t="str">
+      <x:c r="A5" s="28" t="str">
         <x:v>Field key</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="str">
+      <x:c r="B5" s="28" t="str">
         <x:v>Field</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="str">
+      <x:c r="C5" s="28" t="str">
         <x:v>Entry</x:v>
       </x:c>
-      <x:c r="D5" s="13" t="str">
+      <x:c r="D5" s="28" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="E5" s="13" t="str">
+      <x:c r="E5" s="28" t="str">
         <x:v>Evidence state</x:v>
       </x:c>
-      <x:c r="F5" s="13" t="str">
+      <x:c r="F5" s="28" t="str">
         <x:v>Source ref</x:v>
       </x:c>
-      <x:c r="G5" s="13" t="str">
+      <x:c r="G5" s="28" t="str">
         <x:v>Synthetic example</x:v>
       </x:c>
-      <x:c r="H5" s="13" t="str">
+      <x:c r="H5" s="28" t="str">
         <x:v>Entry guidance and required condition</x:v>
       </x:c>
     </x:row>
@@ -3086,11 +3295,11 @@
       <x:c r="B6" s="14" t="str">
         <x:v>Activity instance ID</x:v>
       </x:c>
-      <x:c r="C6" s="19"/>
+      <x:c r="C6" s="29"/>
       <x:c r="D6" s="14" t="str"/>
-      <x:c r="E6" s="15"/>
-      <x:c r="F6" s="15"/>
-      <x:c r="G6" s="17" t="str">
+      <x:c r="E6" s="31"/>
+      <x:c r="F6" s="31"/>
+      <x:c r="G6" s="33" t="str">
         <x:v>SYN-ACTIVITY-001</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
@@ -3104,11 +3313,11 @@
       <x:c r="B7" s="14" t="str">
         <x:v>Estimate alternative ID</x:v>
       </x:c>
-      <x:c r="C7" s="19"/>
+      <x:c r="C7" s="29"/>
       <x:c r="D7" s="14" t="str"/>
-      <x:c r="E7" s="15"/>
-      <x:c r="F7" s="15"/>
-      <x:c r="G7" s="17" t="str">
+      <x:c r="E7" s="31"/>
+      <x:c r="F7" s="31"/>
+      <x:c r="G7" s="33" t="str">
         <x:v>SYN-ALT-A</x:v>
       </x:c>
       <x:c r="H7" s="18" t="str">
@@ -3122,11 +3331,11 @@
       <x:c r="B8" s="14" t="str">
         <x:v>System/line instance ID</x:v>
       </x:c>
-      <x:c r="C8" s="19"/>
+      <x:c r="C8" s="29"/>
       <x:c r="D8" s="14" t="str"/>
-      <x:c r="E8" s="15"/>
-      <x:c r="F8" s="15"/>
-      <x:c r="G8" s="17" t="str">
+      <x:c r="E8" s="31"/>
+      <x:c r="F8" s="31"/>
+      <x:c r="G8" s="33" t="str">
         <x:v>SYN-LINE-001</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
@@ -3140,15 +3349,15 @@
       <x:c r="B9" s="14" t="str">
         <x:v>Exact workbench run ID</x:v>
       </x:c>
-      <x:c r="C9" s="19"/>
+      <x:c r="C9" s="29"/>
       <x:c r="D9" s="14" t="str"/>
-      <x:c r="E9" s="15"/>
-      <x:c r="F9" s="15"/>
-      <x:c r="G9" s="17" t="str">
+      <x:c r="E9" s="31"/>
+      <x:c r="F9" s="31"/>
+      <x:c r="G9" s="33" t="str">
         <x:v>SYN-RUN-001</x:v>
       </x:c>
       <x:c r="H9" s="18" t="str">
-        <x:v>Required. Must match accepted parts/facts.</x:v>
+        <x:v>When workbench-derived. Must match accepted parts/facts.</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="42" customHeight="1">
@@ -3156,15 +3365,15 @@
         <x:v>source_content_hash</x:v>
       </x:c>
       <x:c r="B10" s="14" t="str">
-        <x:v>Run content hash</x:v>
-      </x:c>
-      <x:c r="C10" s="19"/>
+        <x:v>Source content hash</x:v>
+      </x:c>
+      <x:c r="C10" s="29"/>
       <x:c r="D10" s="14" t="str"/>
-      <x:c r="E10" s="15"/>
-      <x:c r="F10" s="15"/>
-      <x:c r="G10" s="17"/>
+      <x:c r="E10" s="31"/>
+      <x:c r="F10" s="31"/>
+      <x:c r="G10" s="33"/>
       <x:c r="H10" s="18" t="str">
-        <x:v>Before receiving. Verified SHA-256, never placeholder.</x:v>
+        <x:v>Before receiving. Exact workbench or saved Manual/project basis hash; never invent a run.</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="42" customHeight="1">
@@ -3174,11 +3383,11 @@
       <x:c r="B11" s="14" t="str">
         <x:v>Profile ID and version</x:v>
       </x:c>
-      <x:c r="C11" s="19"/>
+      <x:c r="C11" s="29"/>
       <x:c r="D11" s="14" t="str"/>
-      <x:c r="E11" s="15"/>
-      <x:c r="F11" s="15"/>
-      <x:c r="G11" s="17" t="str">
+      <x:c r="E11" s="31"/>
+      <x:c r="F11" s="31"/>
+      <x:c r="G11" s="33" t="str">
         <x:v>SYN-PROFILE-001@1</x:v>
       </x:c>
       <x:c r="H11" s="18" t="str">
@@ -3192,11 +3401,11 @@
       <x:c r="B12" s="14" t="str">
         <x:v>Activity standard reference</x:v>
       </x:c>
-      <x:c r="C12" s="19"/>
+      <x:c r="C12" s="29"/>
       <x:c r="D12" s="14" t="str"/>
-      <x:c r="E12" s="15"/>
-      <x:c r="F12" s="15"/>
-      <x:c r="G12" s="17" t="str">
+      <x:c r="E12" s="31"/>
+      <x:c r="F12" s="31"/>
+      <x:c r="G12" s="33" t="str">
         <x:v>SYN-ACT-001@1</x:v>
       </x:c>
       <x:c r="H12" s="18" t="str">
@@ -3210,11 +3419,11 @@
       <x:c r="B13" s="14" t="str">
         <x:v>Applicability</x:v>
       </x:c>
-      <x:c r="C13" s="19"/>
+      <x:c r="C13" s="29"/>
       <x:c r="D13" s="14" t="str"/>
-      <x:c r="E13" s="15"/>
-      <x:c r="F13" s="15"/>
-      <x:c r="G13" s="17" t="str">
+      <x:c r="E13" s="31"/>
+      <x:c r="F13" s="31"/>
+      <x:c r="G13" s="33" t="str">
         <x:v>Applicable</x:v>
       </x:c>
       <x:c r="H13" s="18" t="str">
@@ -3228,11 +3437,11 @@
       <x:c r="B14" s="14" t="str">
         <x:v>Commercial selection</x:v>
       </x:c>
-      <x:c r="C14" s="19"/>
+      <x:c r="C14" s="29"/>
       <x:c r="D14" s="14" t="str"/>
-      <x:c r="E14" s="15"/>
-      <x:c r="F14" s="15"/>
-      <x:c r="G14" s="17" t="str">
+      <x:c r="E14" s="31"/>
+      <x:c r="F14" s="31"/>
+      <x:c r="G14" s="33" t="str">
         <x:v>Base</x:v>
       </x:c>
       <x:c r="H14" s="18" t="str">
@@ -3246,11 +3455,11 @@
       <x:c r="B15" s="14" t="str">
         <x:v>Delivery responsibility</x:v>
       </x:c>
-      <x:c r="C15" s="19"/>
+      <x:c r="C15" s="29"/>
       <x:c r="D15" s="14" t="str"/>
-      <x:c r="E15" s="15"/>
-      <x:c r="F15" s="15"/>
-      <x:c r="G15" s="17" t="str">
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="33" t="str">
         <x:v>Supplier</x:v>
       </x:c>
       <x:c r="H15" s="18" t="str">
@@ -3264,11 +3473,11 @@
       <x:c r="B16" s="14" t="str">
         <x:v>Coverage basis</x:v>
       </x:c>
-      <x:c r="C16" s="19"/>
+      <x:c r="C16" s="29"/>
       <x:c r="D16" s="14" t="str"/>
-      <x:c r="E16" s="15"/>
-      <x:c r="F16" s="15"/>
-      <x:c r="G16" s="17" t="str">
+      <x:c r="E16" s="31"/>
+      <x:c r="F16" s="31"/>
+      <x:c r="G16" s="33" t="str">
         <x:v>SupplierIncluded</x:v>
       </x:c>
       <x:c r="H16" s="18" t="str">
@@ -3282,11 +3491,11 @@
       <x:c r="B17" s="14" t="str">
         <x:v>Coverage evidence/owner</x:v>
       </x:c>
-      <x:c r="C17" s="19"/>
+      <x:c r="C17" s="29"/>
       <x:c r="D17" s="14" t="str"/>
-      <x:c r="E17" s="15"/>
-      <x:c r="F17" s="15"/>
-      <x:c r="G17" s="17" t="str">
+      <x:c r="E17" s="31"/>
+      <x:c r="F17" s="31"/>
+      <x:c r="G17" s="33" t="str">
         <x:v>SYN-SRC-001</x:v>
       </x:c>
       <x:c r="H17" s="18" t="str">
@@ -3300,17 +3509,17 @@
       <x:c r="B18" s="14" t="str">
         <x:v>Effective installed quantity</x:v>
       </x:c>
-      <x:c r="C18" s="20"/>
+      <x:c r="C18" s="38"/>
       <x:c r="D18" s="14" t="str">
         <x:v>driver unit</x:v>
       </x:c>
-      <x:c r="E18" s="15"/>
-      <x:c r="F18" s="15"/>
-      <x:c r="G18" s="21" t="n">
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="37" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="H18" s="18" t="str">
-        <x:v>When calculated. Separate from spares, waste and purchase packs.</x:v>
+        <x:v>For installation quantity basis. Use only with InstalledQuantity and its exact driver unit; leave blank for test/session drivers. Exclude spares and purchase packs.</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="42" customHeight="1">
@@ -3320,12 +3529,12 @@
       <x:c r="B19" s="14" t="str">
         <x:v>Effective driver unit</x:v>
       </x:c>
-      <x:c r="C19" s="19"/>
+      <x:c r="C19" s="29"/>
       <x:c r="D19" s="14" t="str"/>
-      <x:c r="E19" s="15"/>
-      <x:c r="F19" s="15"/>
-      <x:c r="G19" s="17" t="str">
-        <x:v>each</x:v>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="33" t="str">
+        <x:v>test</x:v>
       </x:c>
       <x:c r="H19" s="18" t="str">
         <x:v>When calculated. Exact dimensional basis.</x:v>
@@ -3338,11 +3547,11 @@
       <x:c r="B20" s="14" t="str">
         <x:v>Manual effort basis</x:v>
       </x:c>
-      <x:c r="C20" s="19"/>
+      <x:c r="C20" s="29"/>
       <x:c r="D20" s="14" t="str"/>
-      <x:c r="E20" s="15"/>
-      <x:c r="F20" s="15"/>
-      <x:c r="G20" s="17"/>
+      <x:c r="E20" s="31"/>
+      <x:c r="F20" s="31"/>
+      <x:c r="G20" s="33"/>
       <x:c r="H20" s="18" t="str">
         <x:v>When Manual. Reasoned evidence and applicable review; no silent zero.</x:v>
       </x:c>
@@ -3354,11 +3563,11 @@
       <x:c r="B21" s="14" t="str">
         <x:v>Technical review</x:v>
       </x:c>
-      <x:c r="C21" s="19"/>
+      <x:c r="C21" s="29"/>
       <x:c r="D21" s="14" t="str"/>
-      <x:c r="E21" s="15"/>
-      <x:c r="F21" s="15"/>
-      <x:c r="G21" s="17" t="str">
+      <x:c r="E21" s="31"/>
+      <x:c r="F21" s="31"/>
+      <x:c r="G21" s="33" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="H21" s="18" t="str">
@@ -3372,22 +3581,199 @@
       <x:c r="B22" s="14" t="str">
         <x:v>Commercial scope review</x:v>
       </x:c>
-      <x:c r="C22" s="19"/>
+      <x:c r="C22" s="29"/>
       <x:c r="D22" s="14" t="str"/>
-      <x:c r="E22" s="15"/>
-      <x:c r="F22" s="15"/>
-      <x:c r="G22" s="17" t="str">
+      <x:c r="E22" s="31"/>
+      <x:c r="F22" s="31"/>
+      <x:c r="G22" s="33" t="str">
         <x:v>Pending</x:v>
       </x:c>
       <x:c r="H22" s="18" t="str">
         <x:v>Required. Unknown required responsibility or coverage blocks Use.</x:v>
       </x:c>
     </x:row>
+    <x:row r="23" ht="42" customHeight="1">
+      <x:c r="A23" s="14" t="str">
+        <x:v>company_key</x:v>
+      </x:c>
+      <x:c r="B23" s="14" t="str">
+        <x:v>PPO company key</x:v>
+      </x:c>
+      <x:c r="C23" s="29"/>
+      <x:c r="D23" s="14" t="str"/>
+      <x:c r="E23" s="31"/>
+      <x:c r="F23" s="31"/>
+      <x:c r="G23" s="33" t="str">
+        <x:v>SYN-COMPANY</x:v>
+      </x:c>
+      <x:c r="H23" s="18" t="str">
+        <x:v>Required. Exact company context.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="42" customHeight="1">
+      <x:c r="A24" s="14" t="str">
+        <x:v>workspace_id</x:v>
+      </x:c>
+      <x:c r="B24" s="14" t="str">
+        <x:v>Estimating workspace ID</x:v>
+      </x:c>
+      <x:c r="C24" s="29"/>
+      <x:c r="D24" s="14" t="str"/>
+      <x:c r="E24" s="31"/>
+      <x:c r="F24" s="31"/>
+      <x:c r="G24" s="33" t="str">
+        <x:v>SYN-WORKSPACE</x:v>
+      </x:c>
+      <x:c r="H24" s="18" t="str">
+        <x:v>Required. Exact workspace owning the alternative.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="42" customHeight="1">
+      <x:c r="A25" s="14" t="str">
+        <x:v>scope_revision_id</x:v>
+      </x:c>
+      <x:c r="B25" s="14" t="str">
+        <x:v>Saved scope revision</x:v>
+      </x:c>
+      <x:c r="C25" s="29"/>
+      <x:c r="D25" s="14" t="str"/>
+      <x:c r="E25" s="31"/>
+      <x:c r="F25" s="31"/>
+      <x:c r="G25" s="33" t="str">
+        <x:v>SYN-SCOPE-001</x:v>
+      </x:c>
+      <x:c r="H25" s="18" t="str">
+        <x:v>Before receiving. Immutable Discovery or Express revision.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="42" customHeight="1">
+      <x:c r="A26" s="14" t="str">
+        <x:v>workbench_instance_id</x:v>
+      </x:c>
+      <x:c r="B26" s="14" t="str">
+        <x:v>Source workbench instance</x:v>
+      </x:c>
+      <x:c r="C26" s="29"/>
+      <x:c r="D26" s="14" t="str"/>
+      <x:c r="E26" s="31"/>
+      <x:c r="F26" s="31"/>
+      <x:c r="G26" s="33" t="str">
+        <x:v>SYN-WB-001</x:v>
+      </x:c>
+      <x:c r="H26" s="18" t="str">
+        <x:v>When workbench-derived. Instance identity distinct from system and run; leave blank for project Manual work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="14" t="str">
+        <x:v>driver_key</x:v>
+      </x:c>
+      <x:c r="B27" s="14" t="str">
+        <x:v>Effective driver key</x:v>
+      </x:c>
+      <x:c r="C27" s="29"/>
+      <x:c r="D27" s="14" t="str"/>
+      <x:c r="E27" s="31"/>
+      <x:c r="F27" s="31"/>
+      <x:c r="G27" s="33" t="str">
+        <x:v>commissioning_scenario_count</x:v>
+      </x:c>
+      <x:c r="H27" s="18" t="str">
+        <x:v>When calculated. Use the selected standard driver: installed quantity, trials, sessions or project work.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="14" t="str">
+        <x:v>fact_reference</x:v>
+      </x:c>
+      <x:c r="B28" s="14" t="str">
+        <x:v>Exact fact reference</x:v>
+      </x:c>
+      <x:c r="C28" s="29"/>
+      <x:c r="D28" s="14" t="str"/>
+      <x:c r="E28" s="31"/>
+      <x:c r="F28" s="31"/>
+      <x:c r="G28" s="33" t="str">
+        <x:v>SYN-FACT-001@1</x:v>
+      </x:c>
+      <x:c r="H28" s="18" t="str">
+        <x:v>Before calculation. Exact derived fact ID/version and source; Manual/project basis must be evidenced.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="14" t="str">
+        <x:v>project_exception_reference</x:v>
+      </x:c>
+      <x:c r="B29" s="14" t="str">
+        <x:v>Project profile exception</x:v>
+      </x:c>
+      <x:c r="C29" s="29"/>
+      <x:c r="D29" s="14" t="str"/>
+      <x:c r="E29" s="31"/>
+      <x:c r="F29" s="31"/>
+      <x:c r="G29" s="33"/>
+      <x:c r="H29" s="18" t="str">
+        <x:v>When overridden. Record reviewed project-specific inheritance or coverage exception.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="42" customHeight="1">
+      <x:c r="A30" s="14" t="str">
+        <x:v>scope_source_kind</x:v>
+      </x:c>
+      <x:c r="B30" s="14" t="str">
+        <x:v>Saved scope type</x:v>
+      </x:c>
+      <x:c r="C30" s="29"/>
+      <x:c r="D30" s="14" t="str"/>
+      <x:c r="E30" s="31"/>
+      <x:c r="F30" s="31"/>
+      <x:c r="G30" s="33" t="str">
+        <x:v>Discovery</x:v>
+      </x:c>
+      <x:c r="H30" s="18" t="str">
+        <x:v>Required. Do not fabricate Complete Discovery for Express.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="42" customHeight="1">
+      <x:c r="A31" s="14" t="str">
+        <x:v>quantity_basis</x:v>
+      </x:c>
+      <x:c r="B31" s="14" t="str">
+        <x:v>Effective quantity basis</x:v>
+      </x:c>
+      <x:c r="C31" s="29"/>
+      <x:c r="D31" s="14" t="str"/>
+      <x:c r="E31" s="31"/>
+      <x:c r="F31" s="31"/>
+      <x:c r="G31" s="33" t="str">
+        <x:v>TestCount</x:v>
+      </x:c>
+      <x:c r="H31" s="18" t="str">
+        <x:v>When calculated. Installed quantity is one basis; packs/waste do not automatically drive effort.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="42" customHeight="1">
+      <x:c r="A32" s="14" t="str">
+        <x:v>effective_driver_quantity</x:v>
+      </x:c>
+      <x:c r="B32" s="14" t="str">
+        <x:v>Effective driver quantity</x:v>
+      </x:c>
+      <x:c r="C32" s="38"/>
+      <x:c r="D32" s="14" t="str">
+        <x:v>driver unit</x:v>
+      </x:c>
+      <x:c r="E32" s="31"/>
+      <x:c r="F32" s="31"/>
+      <x:c r="G32" s="37" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="H32" s="18" t="str">
+        <x:v>When calculated. Tests, sessions or installed quantity in the exact driver unit; CPQ resolves the approved value.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
-  <x:dataValidations count="7">
-    <x:dataValidation type="list" sqref="E6:E22">
-      <x:formula1>"Unknown,NotApplicable,Assumed,CustomerAdvised,SupplierDocumented,TrialMeasured"</x:formula1>
-    </x:dataValidation>
+  <x:dataValidations count="9">
     <x:dataValidation type="list" sqref="C13">
       <x:formula1>"Applicable,NotApplicable,Unknown"</x:formula1>
     </x:dataValidation>
@@ -3405,6 +3791,15 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C22">
       <x:formula1>"Pending,Reviewed,Rejected"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E6:E32">
+      <x:formula1>"Unknown,NotApplicable,Assumed,CustomerAdvised,SupplierDocumented,TrialMeasured"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C30">
+      <x:formula1>"Discovery,Express"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="C31">
+      <x:formula1>"InstalledQuantity,TestCount,SessionCount,Project,Manual"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3472,28 +3867,28 @@
       <x:c r="H4" s="7"/>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
-      <x:c r="A5" s="13" t="str">
+      <x:c r="A5" s="28" t="str">
         <x:v>Field key</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="str">
+      <x:c r="B5" s="28" t="str">
         <x:v>Field</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="str">
+      <x:c r="C5" s="28" t="str">
         <x:v>Entry</x:v>
       </x:c>
-      <x:c r="D5" s="13" t="str">
+      <x:c r="D5" s="28" t="str">
         <x:v>Unit</x:v>
       </x:c>
-      <x:c r="E5" s="13" t="str">
+      <x:c r="E5" s="28" t="str">
         <x:v>Evidence state</x:v>
       </x:c>
-      <x:c r="F5" s="13" t="str">
+      <x:c r="F5" s="28" t="str">
         <x:v>Source ref</x:v>
       </x:c>
-      <x:c r="G5" s="13" t="str">
+      <x:c r="G5" s="28" t="str">
         <x:v>Synthetic example</x:v>
       </x:c>
-      <x:c r="H5" s="13" t="str">
+      <x:c r="H5" s="28" t="str">
         <x:v>Entry guidance and required condition</x:v>
       </x:c>
     </x:row>
@@ -3504,11 +3899,11 @@
       <x:c r="B6" s="14" t="str">
         <x:v>Content link ID</x:v>
       </x:c>
-      <x:c r="C6" s="19"/>
+      <x:c r="C6" s="29"/>
       <x:c r="D6" s="14" t="str"/>
-      <x:c r="E6" s="15"/>
-      <x:c r="F6" s="15"/>
-      <x:c r="G6" s="17" t="str">
+      <x:c r="E6" s="31"/>
+      <x:c r="F6" s="31"/>
+      <x:c r="G6" s="33" t="str">
         <x:v>SYN-CONTENT-001</x:v>
       </x:c>
       <x:c r="H6" s="18" t="str">
@@ -3522,11 +3917,11 @@
       <x:c r="B7" s="14" t="str">
         <x:v>Profile ID and version</x:v>
       </x:c>
-      <x:c r="C7" s="19"/>
+      <x:c r="C7" s="29"/>
       <x:c r="D7" s="14" t="str"/>
-      <x:c r="E7" s="15"/>
-      <x:c r="F7" s="15"/>
-      <x:c r="G7" s="17" t="str">
+      <x:c r="E7" s="31"/>
+      <x:c r="F7" s="31"/>
+      <x:c r="G7" s="33" t="str">
         <x:v>SYN-PROFILE-001@1</x:v>
       </x:c>
       <x:c r="H7" s="18" t="str">
@@ -3540,11 +3935,11 @@
       <x:c r="B8" s="14" t="str">
         <x:v>Content clause ID</x:v>
       </x:c>
-      <x:c r="C8" s="19"/>
+      <x:c r="C8" s="29"/>
       <x:c r="D8" s="14" t="str"/>
-      <x:c r="E8" s="15"/>
-      <x:c r="F8" s="15"/>
-      <x:c r="G8" s="17" t="str">
+      <x:c r="E8" s="31"/>
+      <x:c r="F8" s="31"/>
+      <x:c r="G8" s="33" t="str">
         <x:v>SYN-CLAUSE-001</x:v>
       </x:c>
       <x:c r="H8" s="18" t="str">
@@ -3558,11 +3953,11 @@
       <x:c r="B9" s="14" t="str">
         <x:v>Clause version</x:v>
       </x:c>
-      <x:c r="C9" s="19"/>
+      <x:c r="C9" s="29"/>
       <x:c r="D9" s="14" t="str"/>
-      <x:c r="E9" s="15"/>
-      <x:c r="F9" s="15"/>
-      <x:c r="G9" s="17" t="str">
+      <x:c r="E9" s="31"/>
+      <x:c r="F9" s="31"/>
+      <x:c r="G9" s="33" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="H9" s="18" t="str">
@@ -3576,11 +3971,11 @@
       <x:c r="B10" s="14" t="str">
         <x:v>Content category</x:v>
       </x:c>
-      <x:c r="C10" s="19"/>
+      <x:c r="C10" s="29"/>
       <x:c r="D10" s="14" t="str"/>
-      <x:c r="E10" s="15"/>
-      <x:c r="F10" s="15"/>
-      <x:c r="G10" s="17" t="str">
+      <x:c r="E10" s="31"/>
+      <x:c r="F10" s="31"/>
+      <x:c r="G10" s="33" t="str">
         <x:v>Commissioning</x:v>
       </x:c>
       <x:c r="H10" s="18" t="str">
@@ -3594,11 +3989,11 @@
       <x:c r="B11" s="14" t="str">
         <x:v>Audience</x:v>
       </x:c>
-      <x:c r="C11" s="19"/>
+      <x:c r="C11" s="29"/>
       <x:c r="D11" s="14" t="str"/>
-      <x:c r="E11" s="15"/>
-      <x:c r="F11" s="15"/>
-      <x:c r="G11" s="17" t="str">
+      <x:c r="E11" s="31"/>
+      <x:c r="F11" s="31"/>
+      <x:c r="G11" s="33" t="str">
         <x:v>Internal</x:v>
       </x:c>
       <x:c r="H11" s="18" t="str">
@@ -3612,11 +4007,11 @@
       <x:c r="B12" s="14" t="str">
         <x:v>Content applicability</x:v>
       </x:c>
-      <x:c r="C12" s="19"/>
+      <x:c r="C12" s="29"/>
       <x:c r="D12" s="14" t="str"/>
-      <x:c r="E12" s="15"/>
-      <x:c r="F12" s="15"/>
-      <x:c r="G12" s="17" t="str">
+      <x:c r="E12" s="31"/>
+      <x:c r="F12" s="31"/>
+      <x:c r="G12" s="33" t="str">
         <x:v>Selected commissioning with supplier responsibility</x:v>
       </x:c>
       <x:c r="H12" s="18" t="str">
@@ -3630,11 +4025,11 @@
       <x:c r="B13" s="14" t="str">
         <x:v>Quotation package</x:v>
       </x:c>
-      <x:c r="C13" s="19"/>
+      <x:c r="C13" s="29"/>
       <x:c r="D13" s="14" t="str"/>
-      <x:c r="E13" s="15"/>
-      <x:c r="F13" s="15"/>
-      <x:c r="G13" s="17" t="str">
+      <x:c r="E13" s="31"/>
+      <x:c r="F13" s="31"/>
+      <x:c r="G13" s="33" t="str">
         <x:v>SYN-LINE-PACKAGE</x:v>
       </x:c>
       <x:c r="H13" s="18" t="str">
@@ -3648,11 +4043,11 @@
       <x:c r="B14" s="14" t="str">
         <x:v>Deduplication key</x:v>
       </x:c>
-      <x:c r="C14" s="19"/>
+      <x:c r="C14" s="29"/>
       <x:c r="D14" s="14" t="str"/>
-      <x:c r="E14" s="15"/>
-      <x:c r="F14" s="15"/>
-      <x:c r="G14" s="17" t="str">
+      <x:c r="E14" s="31"/>
+      <x:c r="F14" s="31"/>
+      <x:c r="G14" s="33" t="str">
         <x:v>SYN-COMMISSIONING</x:v>
       </x:c>
       <x:c r="H14" s="18" t="str">
@@ -3666,11 +4061,11 @@
       <x:c r="B15" s="14" t="str">
         <x:v>Contradiction group</x:v>
       </x:c>
-      <x:c r="C15" s="19"/>
+      <x:c r="C15" s="29"/>
       <x:c r="D15" s="14" t="str"/>
-      <x:c r="E15" s="15"/>
-      <x:c r="F15" s="15"/>
-      <x:c r="G15" s="17" t="str">
+      <x:c r="E15" s="31"/>
+      <x:c r="F15" s="31"/>
+      <x:c r="G15" s="33" t="str">
         <x:v>SYN-INCLUDE-EXCLUDE</x:v>
       </x:c>
       <x:c r="H15" s="18" t="str">
@@ -3684,11 +4079,11 @@
       <x:c r="B16" s="14" t="str">
         <x:v>Allowed merge fields</x:v>
       </x:c>
-      <x:c r="C16" s="19"/>
+      <x:c r="C16" s="29"/>
       <x:c r="D16" s="14" t="str"/>
-      <x:c r="E16" s="15"/>
-      <x:c r="F16" s="15"/>
-      <x:c r="G16" s="17" t="str">
+      <x:c r="E16" s="31"/>
+      <x:c r="F16" s="31"/>
+      <x:c r="G16" s="33" t="str">
         <x:v>system_name; responsibility</x:v>
       </x:c>
       <x:c r="H16" s="18" t="str">
@@ -3702,11 +4097,11 @@
       <x:c r="B17" s="14" t="str">
         <x:v>Permitted edit policy</x:v>
       </x:c>
-      <x:c r="C17" s="19"/>
+      <x:c r="C17" s="29"/>
       <x:c r="D17" s="14" t="str"/>
-      <x:c r="E17" s="15"/>
-      <x:c r="F17" s="15"/>
-      <x:c r="G17" s="17" t="str">
+      <x:c r="E17" s="31"/>
+      <x:c r="F17" s="31"/>
+      <x:c r="G17" s="33" t="str">
         <x:v>Approved local amendments require review</x:v>
       </x:c>
       <x:c r="H17" s="18" t="str">
@@ -3720,11 +4115,11 @@
       <x:c r="B18" s="14" t="str">
         <x:v>Clause approval state</x:v>
       </x:c>
-      <x:c r="C18" s="19"/>
+      <x:c r="C18" s="29"/>
       <x:c r="D18" s="14" t="str"/>
-      <x:c r="E18" s="15"/>
-      <x:c r="F18" s="15"/>
-      <x:c r="G18" s="17" t="str">
+      <x:c r="E18" s="31"/>
+      <x:c r="F18" s="31"/>
+      <x:c r="G18" s="33" t="str">
         <x:v>Draft</x:v>
       </x:c>
       <x:c r="H18" s="18" t="str">
@@ -3738,20 +4133,69 @@
       <x:c r="B19" s="14" t="str">
         <x:v>Approval evidence</x:v>
       </x:c>
-      <x:c r="C19" s="19"/>
+      <x:c r="C19" s="29"/>
       <x:c r="D19" s="14" t="str"/>
-      <x:c r="E19" s="15"/>
-      <x:c r="F19" s="15"/>
-      <x:c r="G19" s="17"/>
+      <x:c r="E19" s="31"/>
+      <x:c r="F19" s="31"/>
+      <x:c r="G19" s="33"/>
       <x:c r="H19" s="18" t="str">
         <x:v>Before Approved. Actual content owner approval.</x:v>
       </x:c>
     </x:row>
+    <x:row r="20" ht="42" customHeight="1">
+      <x:c r="A20" s="14" t="str">
+        <x:v>content_owner</x:v>
+      </x:c>
+      <x:c r="B20" s="14" t="str">
+        <x:v>Content owner</x:v>
+      </x:c>
+      <x:c r="C20" s="29"/>
+      <x:c r="D20" s="14" t="str"/>
+      <x:c r="E20" s="31"/>
+      <x:c r="F20" s="31"/>
+      <x:c r="G20" s="33"/>
+      <x:c r="H20" s="18" t="str">
+        <x:v>Before quotation. Accountable clause owner from the approved library; not the workbook editor.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="42" customHeight="1">
+      <x:c r="A21" s="14" t="str">
+        <x:v>section_order</x:v>
+      </x:c>
+      <x:c r="B21" s="14" t="str">
+        <x:v>Package section order</x:v>
+      </x:c>
+      <x:c r="C21" s="35"/>
+      <x:c r="D21" s="14" t="str">
+        <x:v>position</x:v>
+      </x:c>
+      <x:c r="E21" s="31"/>
+      <x:c r="F21" s="31"/>
+      <x:c r="G21" s="37" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H21" s="18" t="str">
+        <x:v>Before quotation. Deterministic order within the package; no text-similarity deduplication.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="14" t="str">
+        <x:v>content_hash</x:v>
+      </x:c>
+      <x:c r="B22" s="14" t="str">
+        <x:v>Exact clause content hash</x:v>
+      </x:c>
+      <x:c r="C22" s="29"/>
+      <x:c r="D22" s="14" t="str"/>
+      <x:c r="E22" s="31"/>
+      <x:c r="F22" s="31"/>
+      <x:c r="G22" s="33"/>
+      <x:c r="H22" s="18" t="str">
+        <x:v>Before quotation. Bind approved wording and typed fields from the library; no latest reference.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="E6:E19">
-      <x:formula1>"Unknown,NotApplicable,Assumed,CustomerAdvised,SupplierDocumented,TrialMeasured"</x:formula1>
-    </x:dataValidation>
     <x:dataValidation type="list" sqref="C10">
       <x:formula1>"Installation,Commissioning,Training,Handover,Deliverable,Exclusion,Responsibility,Qualification"</x:formula1>
     </x:dataValidation>
@@ -3760,6 +4204,9 @@
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C18">
       <x:formula1>"Draft,Pending,Approved,Retired"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="E6:E22">
+      <x:formula1>"Unknown,NotApplicable,Assumed,CustomerAdvised,SupplierDocumented,TrialMeasured"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>